<commit_message>
Update document with new changes
</commit_message>
<xml_diff>
--- a/week-1/Ex4A_GTrends.xlsx
+++ b/week-1/Ex4A_GTrends.xlsx
@@ -8,22 +8,38 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JURA\Documents\DataAnalytics\week-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67FE0BB0-5FAA-4DE0-A53B-36AAE6137261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{383DEF25-0B72-4C5D-AAD9-9C17C6D80DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B7DEA57E-16D7-479F-82E1-642219694483}"/>
   </bookViews>
   <sheets>
     <sheet name="GTrends_milkshake_hamburger_202" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="Breakup___2_1_24___2_28_25">GTrends_milkshake_hamburger_202!$G$2:$G$1048576</definedName>
+    <definedName name="Hamburger___2_1_24___2_28_25">GTrends_milkshake_hamburger_202!$D$2:$D$1048576</definedName>
+    <definedName name="Milkshake___2_1_24___2_28_25">GTrends_milkshake_hamburger_202!$E$2:$E$1048576</definedName>
+    <definedName name="Region">GTrends_milkshake_hamburger_202!$B$2:$B$1048576</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
-  <si>
-    <t>Category: All categories</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>Region</t>
   </si>
@@ -188,6 +204,12 @@
   </si>
   <si>
     <t>District of Columbia</t>
+  </si>
+  <si>
+    <t>No: Region</t>
+  </si>
+  <si>
+    <t>Region ID</t>
   </si>
 </sst>
 </file>
@@ -330,7 +352,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -508,6 +530,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -671,9 +699,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -719,7 +748,17 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -730,6 +769,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BAD4BCF4-B24E-4D59-9DFB-948060D6D117}" name="Table1" displayName="Table1" ref="A1:E52" totalsRowShown="0">
+  <autoFilter ref="A1:E52" xr:uid="{BAD4BCF4-B24E-4D59-9DFB-948060D6D117}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:E52">
+    <sortCondition ref="B1:B52"/>
+  </sortState>
+  <tableColumns count="5">
+    <tableColumn id="5" xr3:uid="{DC8C0EC7-F3AA-442A-B314-BC25BBEE1EE1}" name="Region ID"/>
+    <tableColumn id="1" xr3:uid="{99C753F8-B80E-4E77-AFE1-EF7C92D5ED14}" name="Region"/>
+    <tableColumn id="3" xr3:uid="{67691B92-9A11-47A6-8192-5649269FBA84}" name="Hamburger: (2/1/24 - 2/28/25)" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{586A3D8A-5420-47D2-A250-971D60055770}" name="Milkshake: (2/1/24 - 2/28/25)" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{5C3639EE-C712-4FC9-A6CF-EE4949F73B21}" name="Breakup: (2/1/24 - 2/28/25)" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1049,743 +1105,967 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19B08DF5-8E56-4D48-A6EA-17849AC0AB35}">
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.54296875" customWidth="1"/>
+    <col min="5" max="5" width="26.81640625" customWidth="1"/>
+    <col min="6" max="6" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.1796875" customWidth="1"/>
+    <col min="9" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.23</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
       <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.72</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="D3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="1">
-        <v>0.22</v>
+      <c r="B4" t="s">
+        <v>19</v>
       </c>
       <c r="C4" s="1">
         <v>0.67</v>
       </c>
       <c r="D4" s="1">
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+        <v>0.2</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.21</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" s="2">
+        <f>COUNTA(Region)</f>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B5" s="1">
-        <v>0.24</v>
-      </c>
-      <c r="C5" s="1">
-        <v>0.63</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.68</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="B6" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="C6" s="1">
-        <v>0.67</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="1">
-        <v>0.24</v>
-      </c>
-      <c r="C7" s="1">
-        <v>0.63</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="1">
-        <v>0.22</v>
+      <c r="B8" t="s">
+        <v>29</v>
       </c>
       <c r="C8" s="1">
         <v>0.65</v>
       </c>
       <c r="D8" s="1">
+        <v>0.21</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="1">
         <v>0.13</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.17</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="B9" s="1">
-        <v>0.23</v>
-      </c>
-      <c r="C9" s="1">
-        <v>0.65</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.64</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12">
         <v>11</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="D12" s="1">
         <v>0.24</v>
       </c>
-      <c r="C10" s="1">
-        <v>0.64</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="E12" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13">
         <v>12</v>
       </c>
-      <c r="B11" s="1">
-        <v>0.25</v>
-      </c>
-      <c r="C11" s="1">
-        <v>0.62</v>
-      </c>
-      <c r="D11" s="1">
+      <c r="B13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="1">
+        <v>0.73</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E13" s="1">
         <v>0.13</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14">
         <v>13</v>
       </c>
-      <c r="B12" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="C12" s="1">
-        <v>0.65</v>
-      </c>
-      <c r="D12" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="B14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15">
         <v>14</v>
       </c>
-      <c r="B13" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="C13" s="1">
-        <v>0.69</v>
-      </c>
-      <c r="D13" s="1">
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="B15" t="s">
         <v>15</v>
-      </c>
-      <c r="B14" s="1">
-        <v>0.24</v>
-      </c>
-      <c r="C14" s="1">
-        <v>0.62</v>
-      </c>
-      <c r="D14" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="1">
-        <v>0.23</v>
       </c>
       <c r="C15" s="1">
         <v>0.63</v>
       </c>
       <c r="D15" s="1">
+        <v>0.23</v>
+      </c>
+      <c r="E15" s="1">
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0.63</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0.24</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0.68</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18">
         <v>17</v>
       </c>
-      <c r="B16" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="C16" s="1">
-        <v>0.65</v>
-      </c>
-      <c r="D16" s="1">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="1">
-        <v>0.23</v>
-      </c>
-      <c r="C17" s="1">
-        <v>0.63</v>
-      </c>
-      <c r="D17" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="1">
-        <v>0.21</v>
+      <c r="B18" t="s">
+        <v>26</v>
       </c>
       <c r="C18" s="1">
         <v>0.67</v>
       </c>
       <c r="D18" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.68</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E20" s="1">
         <v>0.12</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21">
         <v>20</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="D21" s="1">
+        <v>0.17</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.23</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="D23" s="1">
+        <v>0.21</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0.21</v>
+      </c>
+      <c r="E24" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="1">
+        <v>0.69</v>
+      </c>
+      <c r="D26" s="1">
         <v>0.2</v>
       </c>
-      <c r="C19" s="1">
+      <c r="E26" s="1">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="1">
         <v>0.67</v>
       </c>
-      <c r="D19" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="1">
+      <c r="D27" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="D28" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E28" s="1">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>41</v>
+      </c>
+      <c r="C29" s="1">
+        <v>0.71</v>
+      </c>
+      <c r="D29" s="1">
+        <v>0.17</v>
+      </c>
+      <c r="E29" s="1">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="D30" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E30" s="1">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>45</v>
+      </c>
+      <c r="C31" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="D31" s="1">
+        <v>0.21</v>
+      </c>
+      <c r="E31" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32" s="1">
+        <v>0.61</v>
+      </c>
+      <c r="D32" s="1">
         <v>0.23</v>
       </c>
-      <c r="C20" s="1">
-        <v>0.62</v>
-      </c>
-      <c r="D20" s="1">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="1">
+      <c r="E32" s="1">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="D33" s="1">
         <v>0.21</v>
       </c>
-      <c r="C21" s="1">
-        <v>0.66</v>
-      </c>
-      <c r="D21" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" s="1">
-        <v>0.23</v>
-      </c>
-      <c r="C22" s="1">
-        <v>0.61</v>
-      </c>
-      <c r="D22" s="1">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="C23" s="1">
-        <v>0.67</v>
-      </c>
-      <c r="D23" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="1">
-        <v>0.22</v>
-      </c>
-      <c r="C24" s="1">
-        <v>0.64</v>
-      </c>
-      <c r="D24" s="1">
+      <c r="E33" s="1">
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="1">
-        <v>0.23</v>
-      </c>
-      <c r="C25" s="1">
-        <v>0.64</v>
-      </c>
-      <c r="D25" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" s="1">
-        <v>0.19</v>
-      </c>
-      <c r="C26" s="1">
-        <v>0.67</v>
-      </c>
-      <c r="D26" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="C27" s="1">
-        <v>0.69</v>
-      </c>
-      <c r="D27" s="1">
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="C28" s="1">
-        <v>0.67</v>
-      </c>
-      <c r="D28" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="C29" s="1">
-        <v>0.65</v>
-      </c>
-      <c r="D29" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="1">
-        <v>0.19</v>
-      </c>
-      <c r="C30" s="1">
-        <v>0.67</v>
-      </c>
-      <c r="D30" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31" s="1">
-        <v>0.23</v>
-      </c>
-      <c r="C31" s="1">
-        <v>0.62</v>
-      </c>
-      <c r="D31" s="1">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34">
         <v>33</v>
       </c>
-      <c r="B32" s="1">
-        <v>0.22</v>
-      </c>
-      <c r="C32" s="1">
-        <v>0.64</v>
-      </c>
-      <c r="D32" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>34</v>
-      </c>
-      <c r="B33" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="C33" s="1">
-        <v>0.68</v>
-      </c>
-      <c r="D33" s="1">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" s="1">
-        <v>0.2</v>
+      <c r="B34" t="s">
+        <v>40</v>
       </c>
       <c r="C34" s="1">
         <v>0.62</v>
       </c>
       <c r="D34" s="1">
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+        <v>0.21</v>
+      </c>
+      <c r="E34" s="1">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" s="1">
+        <v>0.63</v>
+      </c>
+      <c r="D35" s="1">
+        <v>0.24</v>
+      </c>
+      <c r="E35" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
         <v>36</v>
-      </c>
-      <c r="B35" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="C35" s="1">
-        <v>0.66</v>
-      </c>
-      <c r="D35" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>37</v>
-      </c>
-      <c r="B36" s="1">
-        <v>0.19</v>
       </c>
       <c r="C36" s="1">
         <v>0.69</v>
       </c>
       <c r="D36" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="E36" s="1">
         <v>0.12</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>17</v>
+      </c>
+      <c r="C37" s="1">
+        <v>0.63</v>
+      </c>
+      <c r="D37" s="1">
+        <v>0.23</v>
+      </c>
+      <c r="E37" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" s="1">
+        <v>0.69</v>
+      </c>
+      <c r="D38" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E38" s="1">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39">
         <v>38</v>
       </c>
-      <c r="B37" s="1">
-        <v>0.19</v>
-      </c>
-      <c r="C37" s="1">
-        <v>0.68</v>
-      </c>
-      <c r="D37" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+      <c r="B39" t="s">
         <v>39</v>
-      </c>
-      <c r="B38" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="C38" s="1">
-        <v>0.65</v>
-      </c>
-      <c r="D38" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>40</v>
-      </c>
-      <c r="B39" s="1">
-        <v>0.18</v>
       </c>
       <c r="C39" s="1">
         <v>0.68</v>
       </c>
       <c r="D39" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="E39" s="1">
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>41</v>
-      </c>
-      <c r="B40" s="1">
-        <v>0.21</v>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>20</v>
       </c>
       <c r="C40" s="1">
         <v>0.62</v>
       </c>
       <c r="D40" s="1">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+        <v>0.23</v>
+      </c>
+      <c r="E40" s="1">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" s="1">
+        <v>0.64</v>
+      </c>
+      <c r="D41" s="1">
+        <v>0.23</v>
+      </c>
+      <c r="E41" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="D42" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="E42" s="1">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43">
         <v>42</v>
       </c>
-      <c r="B41" s="1">
-        <v>0.17</v>
-      </c>
-      <c r="C41" s="1">
-        <v>0.71</v>
-      </c>
-      <c r="D41" s="1">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>43</v>
-      </c>
-      <c r="B42" s="1">
-        <v>0.18</v>
-      </c>
-      <c r="C42" s="1">
-        <v>0.68</v>
-      </c>
-      <c r="D42" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>44</v>
-      </c>
-      <c r="B43" s="1">
-        <v>0.19</v>
+      <c r="B43" t="s">
+        <v>47</v>
       </c>
       <c r="C43" s="1">
-        <v>0.67</v>
+        <v>0.76</v>
       </c>
       <c r="D43" s="1">
         <v>0.14000000000000001</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>45</v>
-      </c>
-      <c r="B44" s="1">
-        <v>0.19</v>
+      <c r="E43" s="1">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>6</v>
       </c>
       <c r="C44" s="1">
         <v>0.67</v>
       </c>
       <c r="D44" s="1">
+        <v>0.21</v>
+      </c>
+      <c r="E44" s="1">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>28</v>
+      </c>
+      <c r="C45" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="D45" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E45" s="1">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="D46" s="1">
+        <v>0.21</v>
+      </c>
+      <c r="E46" s="1">
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47">
         <v>46</v>
       </c>
-      <c r="B45" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="C45" s="1">
-        <v>0.65</v>
-      </c>
-      <c r="D45" s="1">
+      <c r="B47" t="s">
+        <v>50</v>
+      </c>
+      <c r="C47" s="1">
+        <v>0.68</v>
+      </c>
+      <c r="D47" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="E47" s="1">
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48">
         <v>47</v>
       </c>
-      <c r="B46" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="C46" s="1">
-        <v>0.62</v>
-      </c>
-      <c r="D46" s="1">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+      <c r="B48" t="s">
+        <v>24</v>
+      </c>
+      <c r="C48" s="1">
+        <v>0.64</v>
+      </c>
+      <c r="D48" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="E48" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49">
         <v>48</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B49" t="s">
+        <v>43</v>
+      </c>
+      <c r="C49" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="D49" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="E49" s="1">
         <v>0.14000000000000001</v>
       </c>
-      <c r="C47" s="1">
-        <v>0.76</v>
-      </c>
-      <c r="D47" s="1">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50">
         <v>49</v>
       </c>
-      <c r="B48" s="1">
-        <v>0.17</v>
-      </c>
-      <c r="C48" s="1">
-        <v>0.7</v>
-      </c>
-      <c r="D48" s="1">
+      <c r="B50" t="s">
+        <v>10</v>
+      </c>
+      <c r="C50" s="1">
+        <v>0.64</v>
+      </c>
+      <c r="D50" s="1">
+        <v>0.24</v>
+      </c>
+      <c r="E50" s="1">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>35</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="D51" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E51" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>49</v>
+      </c>
+      <c r="C52" s="1">
+        <v>0.71</v>
+      </c>
+      <c r="D52" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="E52" s="1">
         <v>0.13</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>50</v>
-      </c>
-      <c r="B49" s="1">
-        <v>0.16</v>
-      </c>
-      <c r="C49" s="1">
-        <v>0.71</v>
-      </c>
-      <c r="D49" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>51</v>
-      </c>
-      <c r="B50" s="1">
-        <v>0.18</v>
-      </c>
-      <c r="C50" s="1">
-        <v>0.68</v>
-      </c>
-      <c r="D50" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>52</v>
-      </c>
-      <c r="B51" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="C51" s="1">
-        <v>0.73</v>
-      </c>
-      <c r="D51" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>53</v>
-      </c>
-      <c r="B52" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="C52" s="1">
-        <v>0.75</v>
-      </c>
-      <c r="D52" s="1">
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>54</v>
-      </c>
-      <c r="B53" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="C53" s="1">
-        <v>0.72</v>
-      </c>
-      <c r="D53" s="1">
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>55</v>
-      </c>
-      <c r="B54" s="1">
-        <v>0.17</v>
-      </c>
-      <c r="C54" s="1">
-        <v>0.67</v>
-      </c>
-      <c r="D54" s="1">
-        <v>0.16</v>
-      </c>
-    </row>
   </sheetData>
+  <conditionalFormatting sqref="G1:H1">
+    <cfRule type="dataBar" priority="1">
+      <dataBar showValue="0">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{DEA08C32-0F25-4C8D-A6B2-A4EAA8B91309}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+    <cfRule type="dataBar" priority="2">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{06E1442F-AA64-45DA-8F65-2079EBBE9C89}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{DEA08C32-0F25-4C8D-A6B2-A4EAA8B91309}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0" axisPosition="middle">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor theme="3" tint="0.499984740745262"/>
+              <x14:axisColor theme="3" tint="0.499984740745262"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <x14:cfRule type="dataBar" id="{06E1442F-AA64-45DA-8F65-2079EBBE9C89}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>G1:H1</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>